<commit_message>
chg: Added SRNTGT116: Apatitiy Aircraft Factory to JTL
</commit_message>
<xml_diff>
--- a/INTELLIGENCE/OPAC Joint Target List.xlsx
+++ b/INTELLIGENCE/OPAC Joint Target List.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="890" uniqueCount="771">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="895" uniqueCount="774">
   <si>
     <t>OPERATION ARCTIC CITADEL JOINT TARGET LIST</t>
   </si>
@@ -2359,12 +2359,21 @@
   <si>
     <t>Poliarnie Ammunition Factory</t>
   </si>
+  <si>
+    <t>Factory for producing SU-27</t>
+  </si>
+  <si>
+    <t>N67 35.000 E033 24.000</t>
+  </si>
+  <si>
+    <t>Apatity Aircraft Factory</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="33">
+  <fonts count="34">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2376,105 +2385,124 @@
       <sz val="20"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="6"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="8"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFCE9178"/>
       <name val="Consolas"/>
+      <family val="3"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Consolas"/>
+      <family val="3"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFCCCCCC"/>
       <name val="Consolas"/>
+      <family val="3"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -2548,6 +2576,7 @@
       <sz val="11"/>
       <color theme="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -2560,6 +2589,13 @@
       <b/>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -3264,7 +3300,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="170">
+  <cellXfs count="172">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3618,6 +3654,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="45" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3688,9 +3730,7 @@
     <xf numFmtId="0" fontId="17" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="33" fillId="6" borderId="45" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperkobling" xfId="2" builtinId="8"/>
@@ -5086,22 +5126,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="49.5" customHeight="1">
-      <c r="A1" s="135" t="s">
+      <c r="A1" s="137" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="136"/>
-      <c r="C1" s="136"/>
-      <c r="D1" s="136"/>
-      <c r="E1" s="136"/>
-      <c r="F1" s="136"/>
-      <c r="G1" s="137"/>
+      <c r="B1" s="138"/>
+      <c r="C1" s="138"/>
+      <c r="D1" s="138"/>
+      <c r="E1" s="138"/>
+      <c r="F1" s="138"/>
+      <c r="G1" s="139"/>
       <c r="J1"/>
     </row>
     <row r="2" spans="1:10" ht="15.75" thickBot="1">
-      <c r="A2" s="138" t="s">
+      <c r="A2" s="140" t="s">
         <v>739</v>
       </c>
-      <c r="B2" s="139"/>
+      <c r="B2" s="141"/>
       <c r="C2" s="2"/>
       <c r="D2" s="3"/>
       <c r="E2" s="4"/>
@@ -5890,7 +5930,7 @@
       <c r="J37"/>
     </row>
     <row r="38" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A38" s="169" t="s">
+      <c r="A38" s="135" t="s">
         <v>1</v>
       </c>
       <c r="B38" s="127" t="s">
@@ -6726,7 +6766,7 @@
       <c r="J75"/>
     </row>
     <row r="76" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A76" s="169" t="s">
+      <c r="A76" s="135" t="s">
         <v>1</v>
       </c>
       <c r="B76" s="119" t="s">
@@ -8838,7 +8878,7 @@
       <c r="J217"/>
     </row>
     <row r="218" spans="1:10" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A218" s="169" t="s">
+      <c r="A218" s="135" t="s">
         <v>1</v>
       </c>
       <c r="B218" s="119" t="s">
@@ -8950,8 +8990,25 @@
       <c r="J222"/>
     </row>
     <row r="223" spans="1:10" ht="15.75" customHeight="1">
-      <c r="A223" s="6"/>
-      <c r="B223" s="63"/>
+      <c r="A223" s="171" t="s">
+        <v>378</v>
+      </c>
+      <c r="B223" s="104" t="s">
+        <v>773</v>
+      </c>
+      <c r="C223" s="136">
+        <v>9</v>
+      </c>
+      <c r="D223" s="104"/>
+      <c r="E223" s="104" t="s">
+        <v>771</v>
+      </c>
+      <c r="F223" s="104" t="s">
+        <v>772</v>
+      </c>
+      <c r="G223" s="104" t="s">
+        <v>650</v>
+      </c>
       <c r="J223"/>
     </row>
     <row r="224" spans="1:10" ht="15.75" customHeight="1">
@@ -11893,10 +11950,11 @@
     <hyperlink ref="A206" r:id="rId51"/>
     <hyperlink ref="A207" r:id="rId52"/>
     <hyperlink ref="A208" r:id="rId53"/>
+    <hyperlink ref="A223" r:id="rId54"/>
   </hyperlinks>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId54"/>
-  <drawing r:id="rId55"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId55"/>
+  <drawing r:id="rId56"/>
 </worksheet>
 </file>
 
@@ -11918,50 +11976,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="49.5" customHeight="1">
-      <c r="A1" s="140" t="s">
+      <c r="A1" s="142" t="s">
         <v>489</v>
       </c>
-      <c r="B1" s="141"/>
-      <c r="C1" s="141"/>
-      <c r="D1" s="141"/>
-      <c r="E1" s="141"/>
-      <c r="F1" s="141"/>
-      <c r="G1" s="141"/>
-      <c r="H1" s="141"/>
-      <c r="I1" s="142"/>
+      <c r="B1" s="143"/>
+      <c r="C1" s="143"/>
+      <c r="D1" s="143"/>
+      <c r="E1" s="143"/>
+      <c r="F1" s="143"/>
+      <c r="G1" s="143"/>
+      <c r="H1" s="143"/>
+      <c r="I1" s="144"/>
     </row>
     <row r="2" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A2" s="143" t="s">
+      <c r="A2" s="145" t="s">
         <v>490</v>
       </c>
-      <c r="B2" s="144"/>
+      <c r="B2" s="146"/>
       <c r="C2" s="7" t="s">
         <v>491</v>
       </c>
-      <c r="D2" s="145" t="s">
+      <c r="D2" s="147" t="s">
         <v>492</v>
       </c>
-      <c r="E2" s="146"/>
-      <c r="F2" s="146"/>
-      <c r="G2" s="144"/>
-      <c r="H2" s="147" t="s">
+      <c r="E2" s="148"/>
+      <c r="F2" s="148"/>
+      <c r="G2" s="146"/>
+      <c r="H2" s="149" t="s">
         <v>493</v>
       </c>
-      <c r="I2" s="148"/>
+      <c r="I2" s="150"/>
     </row>
     <row r="3" spans="1:17" ht="14.25" customHeight="1"/>
     <row r="4" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A4" s="149" t="s">
+      <c r="A4" s="151" t="s">
         <v>494</v>
       </c>
-      <c r="B4" s="141"/>
-      <c r="C4" s="141"/>
-      <c r="D4" s="141"/>
-      <c r="E4" s="141"/>
-      <c r="F4" s="141"/>
-      <c r="G4" s="141"/>
-      <c r="H4" s="141"/>
-      <c r="I4" s="142"/>
+      <c r="B4" s="143"/>
+      <c r="C4" s="143"/>
+      <c r="D4" s="143"/>
+      <c r="E4" s="143"/>
+      <c r="F4" s="143"/>
+      <c r="G4" s="143"/>
+      <c r="H4" s="143"/>
+      <c r="I4" s="144"/>
     </row>
     <row r="5" spans="1:17" ht="14.25" customHeight="1">
       <c r="A5" s="8" t="s">
@@ -12023,15 +12081,15 @@
       <c r="I6" s="14" t="s">
         <v>511</v>
       </c>
-      <c r="K6" s="150" t="s">
+      <c r="K6" s="152" t="s">
         <v>512</v>
       </c>
-      <c r="L6" s="151"/>
-      <c r="M6" s="151"/>
-      <c r="N6" s="151"/>
-      <c r="O6" s="151"/>
-      <c r="P6" s="151"/>
-      <c r="Q6" s="151"/>
+      <c r="L6" s="153"/>
+      <c r="M6" s="153"/>
+      <c r="N6" s="153"/>
+      <c r="O6" s="153"/>
+      <c r="P6" s="153"/>
+      <c r="Q6" s="153"/>
     </row>
     <row r="7" spans="1:17" ht="14.25" customHeight="1">
       <c r="A7" s="12">
@@ -12061,15 +12119,15 @@
       <c r="I7" s="14" t="s">
         <v>520</v>
       </c>
-      <c r="K7" s="150" t="s">
+      <c r="K7" s="152" t="s">
         <v>521</v>
       </c>
-      <c r="L7" s="151"/>
-      <c r="M7" s="151"/>
-      <c r="N7" s="151"/>
-      <c r="O7" s="151"/>
-      <c r="P7" s="151"/>
-      <c r="Q7" s="151"/>
+      <c r="L7" s="153"/>
+      <c r="M7" s="153"/>
+      <c r="N7" s="153"/>
+      <c r="O7" s="153"/>
+      <c r="P7" s="153"/>
+      <c r="Q7" s="153"/>
     </row>
     <row r="8" spans="1:17" ht="14.25" customHeight="1">
       <c r="A8" s="12">
@@ -12177,17 +12235,17 @@
       <c r="I14" s="18"/>
     </row>
     <row r="15" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A15" s="152" t="s">
+      <c r="A15" s="154" t="s">
         <v>530</v>
       </c>
-      <c r="B15" s="153"/>
-      <c r="C15" s="153"/>
-      <c r="D15" s="153"/>
-      <c r="E15" s="153"/>
-      <c r="F15" s="153"/>
-      <c r="G15" s="153"/>
-      <c r="H15" s="153"/>
-      <c r="I15" s="154"/>
+      <c r="B15" s="155"/>
+      <c r="C15" s="155"/>
+      <c r="D15" s="155"/>
+      <c r="E15" s="155"/>
+      <c r="F15" s="155"/>
+      <c r="G15" s="155"/>
+      <c r="H15" s="155"/>
+      <c r="I15" s="156"/>
     </row>
     <row r="16" spans="1:17" ht="14.25" customHeight="1">
       <c r="A16" s="8" t="s">
@@ -12202,15 +12260,15 @@
       <c r="D16" s="9" t="s">
         <v>502</v>
       </c>
-      <c r="E16" s="155" t="s">
+      <c r="E16" s="157" t="s">
         <v>531</v>
       </c>
-      <c r="F16" s="156"/>
-      <c r="G16" s="155" t="s">
+      <c r="F16" s="158"/>
+      <c r="G16" s="157" t="s">
         <v>532</v>
       </c>
-      <c r="H16" s="157"/>
-      <c r="I16" s="158"/>
+      <c r="H16" s="159"/>
+      <c r="I16" s="160"/>
     </row>
     <row r="17" spans="1:11" ht="14.25" customHeight="1">
       <c r="A17" s="19">
@@ -12225,15 +12283,15 @@
       <c r="D17" s="13" t="s">
         <v>529</v>
       </c>
-      <c r="E17" s="159" t="s">
+      <c r="E17" s="161" t="s">
         <v>534</v>
       </c>
-      <c r="F17" s="156"/>
-      <c r="G17" s="159" t="s">
+      <c r="F17" s="158"/>
+      <c r="G17" s="161" t="s">
         <v>535</v>
       </c>
-      <c r="H17" s="157"/>
-      <c r="I17" s="158"/>
+      <c r="H17" s="159"/>
+      <c r="I17" s="160"/>
     </row>
     <row r="18" spans="1:11" ht="14.25" customHeight="1">
       <c r="A18" s="19">
@@ -12248,15 +12306,15 @@
       <c r="D18" s="13" t="s">
         <v>529</v>
       </c>
-      <c r="E18" s="159" t="s">
+      <c r="E18" s="161" t="s">
         <v>534</v>
       </c>
-      <c r="F18" s="156"/>
-      <c r="G18" s="159" t="s">
+      <c r="F18" s="158"/>
+      <c r="G18" s="161" t="s">
         <v>537</v>
       </c>
-      <c r="H18" s="157"/>
-      <c r="I18" s="158"/>
+      <c r="H18" s="159"/>
+      <c r="I18" s="160"/>
     </row>
     <row r="19" spans="1:11" ht="14.25" customHeight="1">
       <c r="A19" s="19">
@@ -12271,15 +12329,15 @@
       <c r="D19" s="13" t="s">
         <v>539</v>
       </c>
-      <c r="E19" s="159" t="s">
+      <c r="E19" s="161" t="s">
         <v>540</v>
       </c>
-      <c r="F19" s="156"/>
-      <c r="G19" s="159" t="s">
+      <c r="F19" s="158"/>
+      <c r="G19" s="161" t="s">
         <v>541</v>
       </c>
-      <c r="H19" s="157"/>
-      <c r="I19" s="158"/>
+      <c r="H19" s="159"/>
+      <c r="I19" s="160"/>
       <c r="K19" s="11" t="s">
         <v>542</v>
       </c>
@@ -12291,11 +12349,11 @@
       <c r="B20" s="20"/>
       <c r="C20" s="20"/>
       <c r="D20" s="20"/>
-      <c r="E20" s="160"/>
-      <c r="F20" s="156"/>
-      <c r="G20" s="160"/>
-      <c r="H20" s="157"/>
-      <c r="I20" s="158"/>
+      <c r="E20" s="162"/>
+      <c r="F20" s="158"/>
+      <c r="G20" s="162"/>
+      <c r="H20" s="159"/>
+      <c r="I20" s="160"/>
     </row>
     <row r="21" spans="1:11" ht="14.25" customHeight="1">
       <c r="A21" s="19">
@@ -12304,11 +12362,11 @@
       <c r="B21" s="20"/>
       <c r="C21" s="20"/>
       <c r="D21" s="20"/>
-      <c r="E21" s="160"/>
-      <c r="F21" s="156"/>
-      <c r="G21" s="160"/>
-      <c r="H21" s="157"/>
-      <c r="I21" s="158"/>
+      <c r="E21" s="162"/>
+      <c r="F21" s="158"/>
+      <c r="G21" s="162"/>
+      <c r="H21" s="159"/>
+      <c r="I21" s="160"/>
       <c r="K21" s="11" t="s">
         <v>543</v>
       </c>
@@ -12320,11 +12378,11 @@
       <c r="B22" s="20"/>
       <c r="C22" s="20"/>
       <c r="D22" s="20"/>
-      <c r="E22" s="160"/>
-      <c r="F22" s="156"/>
-      <c r="G22" s="160"/>
-      <c r="H22" s="157"/>
-      <c r="I22" s="158"/>
+      <c r="E22" s="162"/>
+      <c r="F22" s="158"/>
+      <c r="G22" s="162"/>
+      <c r="H22" s="159"/>
+      <c r="I22" s="160"/>
     </row>
     <row r="23" spans="1:11" ht="14.25" customHeight="1">
       <c r="A23" s="19">
@@ -12333,11 +12391,11 @@
       <c r="B23" s="20"/>
       <c r="C23" s="20"/>
       <c r="D23" s="20"/>
-      <c r="E23" s="160"/>
-      <c r="F23" s="156"/>
-      <c r="G23" s="160"/>
-      <c r="H23" s="157"/>
-      <c r="I23" s="158"/>
+      <c r="E23" s="162"/>
+      <c r="F23" s="158"/>
+      <c r="G23" s="162"/>
+      <c r="H23" s="159"/>
+      <c r="I23" s="160"/>
     </row>
     <row r="24" spans="1:11" ht="14.25" customHeight="1">
       <c r="A24" s="19">
@@ -12346,11 +12404,11 @@
       <c r="B24" s="20"/>
       <c r="C24" s="20"/>
       <c r="D24" s="20"/>
-      <c r="E24" s="160"/>
-      <c r="F24" s="156"/>
-      <c r="G24" s="160"/>
-      <c r="H24" s="157"/>
-      <c r="I24" s="158"/>
+      <c r="E24" s="162"/>
+      <c r="F24" s="158"/>
+      <c r="G24" s="162"/>
+      <c r="H24" s="159"/>
+      <c r="I24" s="160"/>
     </row>
     <row r="25" spans="1:11" ht="14.25" customHeight="1">
       <c r="A25" s="19">
@@ -12359,11 +12417,11 @@
       <c r="B25" s="20"/>
       <c r="C25" s="20"/>
       <c r="D25" s="20"/>
-      <c r="E25" s="160"/>
-      <c r="F25" s="156"/>
-      <c r="G25" s="160"/>
-      <c r="H25" s="157"/>
-      <c r="I25" s="158"/>
+      <c r="E25" s="162"/>
+      <c r="F25" s="158"/>
+      <c r="G25" s="162"/>
+      <c r="H25" s="159"/>
+      <c r="I25" s="160"/>
     </row>
     <row r="26" spans="1:11" ht="14.25" customHeight="1">
       <c r="A26" s="21">
@@ -12372,11 +12430,11 @@
       <c r="B26" s="16"/>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
-      <c r="E26" s="161"/>
-      <c r="F26" s="144"/>
-      <c r="G26" s="161"/>
-      <c r="H26" s="146"/>
-      <c r="I26" s="148"/>
+      <c r="E26" s="163"/>
+      <c r="F26" s="146"/>
+      <c r="G26" s="163"/>
+      <c r="H26" s="148"/>
+      <c r="I26" s="150"/>
     </row>
     <row r="27" spans="1:11" ht="14.25" customHeight="1"/>
     <row r="28" spans="1:11" ht="14.25" customHeight="1"/>
@@ -13428,11 +13486,11 @@
       <c r="O1" s="25"/>
     </row>
     <row r="2" spans="1:21" ht="14.25" customHeight="1">
-      <c r="A2" s="162" t="s">
+      <c r="A2" s="164" t="s">
         <v>546</v>
       </c>
-      <c r="B2" s="163"/>
-      <c r="C2" s="164"/>
+      <c r="B2" s="165"/>
+      <c r="C2" s="166"/>
       <c r="D2" s="26"/>
       <c r="E2" s="27"/>
       <c r="F2" s="28"/>
@@ -16521,10 +16579,10 @@
   <sheetData>
     <row r="1" spans="2:15" ht="14.25" customHeight="1"/>
     <row r="2" spans="2:15" ht="14.25" customHeight="1">
-      <c r="B2" s="165" t="s">
+      <c r="B2" s="167" t="s">
         <v>554</v>
       </c>
-      <c r="C2" s="156"/>
+      <c r="C2" s="158"/>
       <c r="O2" s="11" t="s">
         <v>555</v>
       </c>
@@ -17735,56 +17793,56 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A3" s="165" t="s">
+      <c r="A3" s="167" t="s">
         <v>587</v>
       </c>
-      <c r="B3" s="157"/>
-      <c r="C3" s="156"/>
+      <c r="B3" s="159"/>
+      <c r="C3" s="158"/>
     </row>
     <row r="4" spans="1:10" ht="14.25" customHeight="1">
       <c r="A4" s="43" t="s">
         <v>495</v>
       </c>
-      <c r="B4" s="167" t="s">
+      <c r="B4" s="169" t="s">
         <v>588</v>
       </c>
-      <c r="C4" s="156"/>
+      <c r="C4" s="158"/>
     </row>
     <row r="5" spans="1:10" ht="96" customHeight="1">
       <c r="A5" s="44" t="s">
         <v>589</v>
       </c>
-      <c r="B5" s="166" t="s">
+      <c r="B5" s="168" t="s">
         <v>590</v>
       </c>
-      <c r="C5" s="156"/>
+      <c r="C5" s="158"/>
     </row>
     <row r="6" spans="1:10" ht="64.5" customHeight="1">
       <c r="A6" s="44" t="s">
         <v>591</v>
       </c>
-      <c r="B6" s="166" t="s">
+      <c r="B6" s="168" t="s">
         <v>592</v>
       </c>
-      <c r="C6" s="156"/>
+      <c r="C6" s="158"/>
     </row>
     <row r="7" spans="1:10" ht="67.5" customHeight="1">
       <c r="A7" s="44" t="s">
         <v>593</v>
       </c>
-      <c r="B7" s="166" t="s">
+      <c r="B7" s="168" t="s">
         <v>594</v>
       </c>
-      <c r="C7" s="156"/>
+      <c r="C7" s="158"/>
     </row>
     <row r="8" spans="1:10" ht="72.75" customHeight="1">
       <c r="A8" s="44" t="s">
         <v>595</v>
       </c>
-      <c r="B8" s="166" t="s">
+      <c r="B8" s="168" t="s">
         <v>596</v>
       </c>
-      <c r="C8" s="156"/>
+      <c r="C8" s="158"/>
     </row>
     <row r="9" spans="1:10" ht="14.25" customHeight="1"/>
     <row r="10" spans="1:10" ht="14.25" customHeight="1"/>
@@ -18809,11 +18867,11 @@
       <c r="D1" s="45"/>
     </row>
     <row r="2" spans="2:10" ht="14.25" customHeight="1">
-      <c r="B2" s="168" t="s">
+      <c r="B2" s="170" t="s">
         <v>597</v>
       </c>
-      <c r="C2" s="141"/>
-      <c r="D2" s="142"/>
+      <c r="C2" s="143"/>
+      <c r="D2" s="144"/>
       <c r="J2" s="11" t="s">
         <v>555</v>
       </c>
@@ -22954,11 +23012,11 @@
     <row r="3" spans="1:10" ht="14.25" customHeight="1"/>
     <row r="4" spans="1:10" ht="14.25" customHeight="1"/>
     <row r="5" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A5" s="167" t="s">
+      <c r="A5" s="169" t="s">
         <v>630</v>
       </c>
-      <c r="B5" s="157"/>
-      <c r="C5" s="156"/>
+      <c r="B5" s="159"/>
+      <c r="C5" s="158"/>
     </row>
     <row r="6" spans="1:10" ht="14.25" customHeight="1">
       <c r="A6" s="43" t="s">

</xml_diff>

<commit_message>
chg: Updated tgt list with SRNTGT069 (3rd Corps HQ) for engagement on D4.2
</commit_message>
<xml_diff>
--- a/INTELLIGENCE/OPAC Joint Target List.xlsx
+++ b/INTELLIGENCE/OPAC Joint Target List.xlsx
@@ -3660,6 +3660,7 @@
     <xf numFmtId="0" fontId="22" fillId="6" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="33" fillId="6" borderId="45" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3669,25 +3670,20 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -3701,17 +3697,22 @@
     <xf numFmtId="0" fontId="10" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3730,7 +3731,6 @@
     <xf numFmtId="0" fontId="17" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="6" borderId="45" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperkobling" xfId="2" builtinId="8"/>
@@ -3765,7 +3765,7 @@
         <xdr:cNvPr id="2" name="image1.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3799,7 +3799,7 @@
         <xdr:cNvPr id="3" name="image2.png" descr="JFACC symbol.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3838,7 +3838,7 @@
         <xdr:cNvPr id="2" name="image3.png" descr="Patch_wip3.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0100-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3872,7 +3872,7 @@
         <xdr:cNvPr id="3" name="image5.png" descr="OPAR JFACC logo.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0100-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3911,7 +3911,7 @@
         <xdr:cNvPr id="2" name="image10.png" descr="Patch_wip3.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0200-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3945,7 +3945,7 @@
         <xdr:cNvPr id="3" name="image5.png" descr="OPAR JFACC logo.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0200-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3984,7 +3984,7 @@
         <xdr:cNvPr id="3" name="Shape 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0300-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4141,7 +4141,7 @@
         <xdr:cNvPr id="4" name="image4.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0300-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4175,7 +4175,7 @@
         <xdr:cNvPr id="5" name="image6.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000005000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0300-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4214,7 +4214,7 @@
         <xdr:cNvPr id="4" name="Shape 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0400-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4371,7 +4371,7 @@
         <xdr:cNvPr id="3" name="image8.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0400-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4405,7 +4405,7 @@
         <xdr:cNvPr id="5" name="image9.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000005000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0400-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4444,7 +4444,7 @@
         <xdr:cNvPr id="5" name="Shape 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000005000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0500-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4625,7 +4625,7 @@
         <xdr:cNvPr id="3" name="image7.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0500-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4659,7 +4659,7 @@
         <xdr:cNvPr id="4" name="image14.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0500-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4698,7 +4698,7 @@
         <xdr:cNvPr id="6" name="Shape 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000006000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0700-000006000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4819,7 +4819,7 @@
         <xdr:cNvPr id="3" name="image13.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0700-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4853,7 +4853,7 @@
         <xdr:cNvPr id="4" name="image11.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0700-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4887,7 +4887,7 @@
         <xdr:cNvPr id="5" name="image12.png">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000005000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0700-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5126,22 +5126,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="49.5" customHeight="1">
-      <c r="A1" s="137" t="s">
+      <c r="A1" s="138" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="138"/>
-      <c r="C1" s="138"/>
-      <c r="D1" s="138"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="138"/>
-      <c r="G1" s="139"/>
+      <c r="B1" s="139"/>
+      <c r="C1" s="139"/>
+      <c r="D1" s="139"/>
+      <c r="E1" s="139"/>
+      <c r="F1" s="139"/>
+      <c r="G1" s="140"/>
       <c r="J1"/>
     </row>
     <row r="2" spans="1:10" ht="15.75" thickBot="1">
-      <c r="A2" s="140" t="s">
+      <c r="A2" s="141" t="s">
         <v>739</v>
       </c>
-      <c r="B2" s="141"/>
+      <c r="B2" s="142"/>
       <c r="C2" s="2"/>
       <c r="D2" s="3"/>
       <c r="E2" s="4"/>
@@ -6702,7 +6702,7 @@
       <c r="J72"/>
     </row>
     <row r="73" spans="1:10" ht="15.75" customHeight="1">
-      <c r="A73" s="106" t="s">
+      <c r="A73" s="134" t="s">
         <v>252</v>
       </c>
       <c r="B73" s="74" t="s">
@@ -8990,7 +8990,7 @@
       <c r="J222"/>
     </row>
     <row r="223" spans="1:10" ht="15.75" customHeight="1">
-      <c r="A223" s="171" t="s">
+      <c r="A223" s="137" t="s">
         <v>378</v>
       </c>
       <c r="B223" s="104" t="s">
@@ -11951,10 +11951,11 @@
     <hyperlink ref="A207" r:id="rId52"/>
     <hyperlink ref="A208" r:id="rId53"/>
     <hyperlink ref="A223" r:id="rId54"/>
+    <hyperlink ref="A73" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId55"/>
-  <drawing r:id="rId56"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId56"/>
+  <drawing r:id="rId57"/>
 </worksheet>
 </file>
 
@@ -11976,50 +11977,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="49.5" customHeight="1">
-      <c r="A1" s="142" t="s">
+      <c r="A1" s="158" t="s">
         <v>489</v>
       </c>
-      <c r="B1" s="143"/>
-      <c r="C1" s="143"/>
-      <c r="D1" s="143"/>
-      <c r="E1" s="143"/>
-      <c r="F1" s="143"/>
-      <c r="G1" s="143"/>
-      <c r="H1" s="143"/>
-      <c r="I1" s="144"/>
+      <c r="B1" s="159"/>
+      <c r="C1" s="159"/>
+      <c r="D1" s="159"/>
+      <c r="E1" s="159"/>
+      <c r="F1" s="159"/>
+      <c r="G1" s="159"/>
+      <c r="H1" s="159"/>
+      <c r="I1" s="160"/>
     </row>
     <row r="2" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A2" s="145" t="s">
+      <c r="A2" s="161" t="s">
         <v>490</v>
       </c>
       <c r="B2" s="146"/>
       <c r="C2" s="7" t="s">
         <v>491</v>
       </c>
-      <c r="D2" s="147" t="s">
+      <c r="D2" s="162" t="s">
         <v>492</v>
       </c>
-      <c r="E2" s="148"/>
-      <c r="F2" s="148"/>
+      <c r="E2" s="149"/>
+      <c r="F2" s="149"/>
       <c r="G2" s="146"/>
-      <c r="H2" s="149" t="s">
+      <c r="H2" s="163" t="s">
         <v>493</v>
       </c>
       <c r="I2" s="150"/>
     </row>
     <row r="3" spans="1:17" ht="14.25" customHeight="1"/>
     <row r="4" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A4" s="151" t="s">
+      <c r="A4" s="164" t="s">
         <v>494</v>
       </c>
-      <c r="B4" s="143"/>
-      <c r="C4" s="143"/>
-      <c r="D4" s="143"/>
-      <c r="E4" s="143"/>
-      <c r="F4" s="143"/>
-      <c r="G4" s="143"/>
-      <c r="H4" s="143"/>
-      <c r="I4" s="144"/>
+      <c r="B4" s="159"/>
+      <c r="C4" s="159"/>
+      <c r="D4" s="159"/>
+      <c r="E4" s="159"/>
+      <c r="F4" s="159"/>
+      <c r="G4" s="159"/>
+      <c r="H4" s="159"/>
+      <c r="I4" s="160"/>
     </row>
     <row r="5" spans="1:17" ht="14.25" customHeight="1">
       <c r="A5" s="8" t="s">
@@ -12263,12 +12264,12 @@
       <c r="E16" s="157" t="s">
         <v>531</v>
       </c>
-      <c r="F16" s="158"/>
+      <c r="F16" s="144"/>
       <c r="G16" s="157" t="s">
         <v>532</v>
       </c>
-      <c r="H16" s="159"/>
-      <c r="I16" s="160"/>
+      <c r="H16" s="147"/>
+      <c r="I16" s="148"/>
     </row>
     <row r="17" spans="1:11" ht="14.25" customHeight="1">
       <c r="A17" s="19">
@@ -12283,15 +12284,15 @@
       <c r="D17" s="13" t="s">
         <v>529</v>
       </c>
-      <c r="E17" s="161" t="s">
+      <c r="E17" s="151" t="s">
         <v>534</v>
       </c>
-      <c r="F17" s="158"/>
-      <c r="G17" s="161" t="s">
+      <c r="F17" s="144"/>
+      <c r="G17" s="151" t="s">
         <v>535</v>
       </c>
-      <c r="H17" s="159"/>
-      <c r="I17" s="160"/>
+      <c r="H17" s="147"/>
+      <c r="I17" s="148"/>
     </row>
     <row r="18" spans="1:11" ht="14.25" customHeight="1">
       <c r="A18" s="19">
@@ -12306,15 +12307,15 @@
       <c r="D18" s="13" t="s">
         <v>529</v>
       </c>
-      <c r="E18" s="161" t="s">
+      <c r="E18" s="151" t="s">
         <v>534</v>
       </c>
-      <c r="F18" s="158"/>
-      <c r="G18" s="161" t="s">
+      <c r="F18" s="144"/>
+      <c r="G18" s="151" t="s">
         <v>537</v>
       </c>
-      <c r="H18" s="159"/>
-      <c r="I18" s="160"/>
+      <c r="H18" s="147"/>
+      <c r="I18" s="148"/>
     </row>
     <row r="19" spans="1:11" ht="14.25" customHeight="1">
       <c r="A19" s="19">
@@ -12329,15 +12330,15 @@
       <c r="D19" s="13" t="s">
         <v>539</v>
       </c>
-      <c r="E19" s="161" t="s">
+      <c r="E19" s="151" t="s">
         <v>540</v>
       </c>
-      <c r="F19" s="158"/>
-      <c r="G19" s="161" t="s">
+      <c r="F19" s="144"/>
+      <c r="G19" s="151" t="s">
         <v>541</v>
       </c>
-      <c r="H19" s="159"/>
-      <c r="I19" s="160"/>
+      <c r="H19" s="147"/>
+      <c r="I19" s="148"/>
       <c r="K19" s="11" t="s">
         <v>542</v>
       </c>
@@ -12349,11 +12350,11 @@
       <c r="B20" s="20"/>
       <c r="C20" s="20"/>
       <c r="D20" s="20"/>
-      <c r="E20" s="162"/>
-      <c r="F20" s="158"/>
-      <c r="G20" s="162"/>
-      <c r="H20" s="159"/>
-      <c r="I20" s="160"/>
+      <c r="E20" s="143"/>
+      <c r="F20" s="144"/>
+      <c r="G20" s="143"/>
+      <c r="H20" s="147"/>
+      <c r="I20" s="148"/>
     </row>
     <row r="21" spans="1:11" ht="14.25" customHeight="1">
       <c r="A21" s="19">
@@ -12362,11 +12363,11 @@
       <c r="B21" s="20"/>
       <c r="C21" s="20"/>
       <c r="D21" s="20"/>
-      <c r="E21" s="162"/>
-      <c r="F21" s="158"/>
-      <c r="G21" s="162"/>
-      <c r="H21" s="159"/>
-      <c r="I21" s="160"/>
+      <c r="E21" s="143"/>
+      <c r="F21" s="144"/>
+      <c r="G21" s="143"/>
+      <c r="H21" s="147"/>
+      <c r="I21" s="148"/>
       <c r="K21" s="11" t="s">
         <v>543</v>
       </c>
@@ -12378,11 +12379,11 @@
       <c r="B22" s="20"/>
       <c r="C22" s="20"/>
       <c r="D22" s="20"/>
-      <c r="E22" s="162"/>
-      <c r="F22" s="158"/>
-      <c r="G22" s="162"/>
-      <c r="H22" s="159"/>
-      <c r="I22" s="160"/>
+      <c r="E22" s="143"/>
+      <c r="F22" s="144"/>
+      <c r="G22" s="143"/>
+      <c r="H22" s="147"/>
+      <c r="I22" s="148"/>
     </row>
     <row r="23" spans="1:11" ht="14.25" customHeight="1">
       <c r="A23" s="19">
@@ -12391,11 +12392,11 @@
       <c r="B23" s="20"/>
       <c r="C23" s="20"/>
       <c r="D23" s="20"/>
-      <c r="E23" s="162"/>
-      <c r="F23" s="158"/>
-      <c r="G23" s="162"/>
-      <c r="H23" s="159"/>
-      <c r="I23" s="160"/>
+      <c r="E23" s="143"/>
+      <c r="F23" s="144"/>
+      <c r="G23" s="143"/>
+      <c r="H23" s="147"/>
+      <c r="I23" s="148"/>
     </row>
     <row r="24" spans="1:11" ht="14.25" customHeight="1">
       <c r="A24" s="19">
@@ -12404,11 +12405,11 @@
       <c r="B24" s="20"/>
       <c r="C24" s="20"/>
       <c r="D24" s="20"/>
-      <c r="E24" s="162"/>
-      <c r="F24" s="158"/>
-      <c r="G24" s="162"/>
-      <c r="H24" s="159"/>
-      <c r="I24" s="160"/>
+      <c r="E24" s="143"/>
+      <c r="F24" s="144"/>
+      <c r="G24" s="143"/>
+      <c r="H24" s="147"/>
+      <c r="I24" s="148"/>
     </row>
     <row r="25" spans="1:11" ht="14.25" customHeight="1">
       <c r="A25" s="19">
@@ -12417,11 +12418,11 @@
       <c r="B25" s="20"/>
       <c r="C25" s="20"/>
       <c r="D25" s="20"/>
-      <c r="E25" s="162"/>
-      <c r="F25" s="158"/>
-      <c r="G25" s="162"/>
-      <c r="H25" s="159"/>
-      <c r="I25" s="160"/>
+      <c r="E25" s="143"/>
+      <c r="F25" s="144"/>
+      <c r="G25" s="143"/>
+      <c r="H25" s="147"/>
+      <c r="I25" s="148"/>
     </row>
     <row r="26" spans="1:11" ht="14.25" customHeight="1">
       <c r="A26" s="21">
@@ -12430,10 +12431,10 @@
       <c r="B26" s="16"/>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
-      <c r="E26" s="163"/>
+      <c r="E26" s="145"/>
       <c r="F26" s="146"/>
-      <c r="G26" s="163"/>
-      <c r="H26" s="148"/>
+      <c r="G26" s="145"/>
+      <c r="H26" s="149"/>
       <c r="I26" s="150"/>
     </row>
     <row r="27" spans="1:11" ht="14.25" customHeight="1"/>
@@ -13412,14 +13413,16 @@
     <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="K6:Q6"/>
+    <mergeCell ref="K7:Q7"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="G16:I16"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="G17:I17"/>
     <mergeCell ref="E18:F18"/>
@@ -13432,16 +13435,14 @@
     <mergeCell ref="E21:F21"/>
     <mergeCell ref="G21:I21"/>
     <mergeCell ref="G22:I22"/>
-    <mergeCell ref="K6:Q6"/>
-    <mergeCell ref="K7:Q7"/>
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="D2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="G26:I26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -13486,11 +13487,11 @@
       <c r="O1" s="25"/>
     </row>
     <row r="2" spans="1:21" ht="14.25" customHeight="1">
-      <c r="A2" s="164" t="s">
+      <c r="A2" s="165" t="s">
         <v>546</v>
       </c>
-      <c r="B2" s="165"/>
-      <c r="C2" s="166"/>
+      <c r="B2" s="166"/>
+      <c r="C2" s="167"/>
       <c r="D2" s="26"/>
       <c r="E2" s="27"/>
       <c r="F2" s="28"/>
@@ -16579,10 +16580,10 @@
   <sheetData>
     <row r="1" spans="2:15" ht="14.25" customHeight="1"/>
     <row r="2" spans="2:15" ht="14.25" customHeight="1">
-      <c r="B2" s="167" t="s">
+      <c r="B2" s="168" t="s">
         <v>554</v>
       </c>
-      <c r="C2" s="158"/>
+      <c r="C2" s="144"/>
       <c r="O2" s="11" t="s">
         <v>555</v>
       </c>
@@ -17793,56 +17794,56 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A3" s="167" t="s">
+      <c r="A3" s="168" t="s">
         <v>587</v>
       </c>
-      <c r="B3" s="159"/>
-      <c r="C3" s="158"/>
+      <c r="B3" s="147"/>
+      <c r="C3" s="144"/>
     </row>
     <row r="4" spans="1:10" ht="14.25" customHeight="1">
       <c r="A4" s="43" t="s">
         <v>495</v>
       </c>
-      <c r="B4" s="169" t="s">
+      <c r="B4" s="170" t="s">
         <v>588</v>
       </c>
-      <c r="C4" s="158"/>
+      <c r="C4" s="144"/>
     </row>
     <row r="5" spans="1:10" ht="96" customHeight="1">
       <c r="A5" s="44" t="s">
         <v>589</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="169" t="s">
         <v>590</v>
       </c>
-      <c r="C5" s="158"/>
+      <c r="C5" s="144"/>
     </row>
     <row r="6" spans="1:10" ht="64.5" customHeight="1">
       <c r="A6" s="44" t="s">
         <v>591</v>
       </c>
-      <c r="B6" s="168" t="s">
+      <c r="B6" s="169" t="s">
         <v>592</v>
       </c>
-      <c r="C6" s="158"/>
+      <c r="C6" s="144"/>
     </row>
     <row r="7" spans="1:10" ht="67.5" customHeight="1">
       <c r="A7" s="44" t="s">
         <v>593</v>
       </c>
-      <c r="B7" s="168" t="s">
+      <c r="B7" s="169" t="s">
         <v>594</v>
       </c>
-      <c r="C7" s="158"/>
+      <c r="C7" s="144"/>
     </row>
     <row r="8" spans="1:10" ht="72.75" customHeight="1">
       <c r="A8" s="44" t="s">
         <v>595</v>
       </c>
-      <c r="B8" s="168" t="s">
+      <c r="B8" s="169" t="s">
         <v>596</v>
       </c>
-      <c r="C8" s="158"/>
+      <c r="C8" s="144"/>
     </row>
     <row r="9" spans="1:10" ht="14.25" customHeight="1"/>
     <row r="10" spans="1:10" ht="14.25" customHeight="1"/>
@@ -18867,11 +18868,11 @@
       <c r="D1" s="45"/>
     </row>
     <row r="2" spans="2:10" ht="14.25" customHeight="1">
-      <c r="B2" s="170" t="s">
+      <c r="B2" s="171" t="s">
         <v>597</v>
       </c>
-      <c r="C2" s="143"/>
-      <c r="D2" s="144"/>
+      <c r="C2" s="159"/>
+      <c r="D2" s="160"/>
       <c r="J2" s="11" t="s">
         <v>555</v>
       </c>
@@ -23012,11 +23013,11 @@
     <row r="3" spans="1:10" ht="14.25" customHeight="1"/>
     <row r="4" spans="1:10" ht="14.25" customHeight="1"/>
     <row r="5" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A5" s="169" t="s">
+      <c r="A5" s="170" t="s">
         <v>630</v>
       </c>
-      <c r="B5" s="159"/>
-      <c r="C5" s="158"/>
+      <c r="B5" s="147"/>
+      <c r="C5" s="144"/>
     </row>
     <row r="6" spans="1:10" ht="14.25" customHeight="1">
       <c r="A6" s="43" t="s">

</xml_diff>